<commit_message>
feat: add Australia price tracker, weekly Pan-EU & Swiss updates (W34-W37), and fast sync engines
</commit_message>
<xml_diff>
--- a/data/price tracker_EU_2026 0814_v1.xlsx
+++ b/data/price tracker_EU_2026 0814_v1.xlsx
@@ -14795,7 +14795,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -15029,7 +15029,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -15107,7 +15107,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -15692,7 +15692,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -15809,7 +15809,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -15848,7 +15848,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -16199,7 +16199,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -16277,7 +16277,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -16316,7 +16316,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -16472,7 +16472,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -16550,7 +16550,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -16667,7 +16667,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -16745,7 +16745,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Free SoundSuite/Soundbar with LG OLED TV 2026 Purchase</t>
         </is>
       </c>
     </row>
@@ -52727,7 +52727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M132"/>
+  <dimension ref="A1:M130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59631,112 +59631,6 @@
       <c r="M130" t="inlineStr">
         <is>
           <t>ISY ILG-2000 LED hangulatvilágítás, 2,2 méter, 2xAA, melegfehér (2V225379)</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Lg</t>
-        </is>
-      </c>
-      <c r="B131" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>OLED G4</t>
-        </is>
-      </c>
-      <c r="D131" t="n">
-        <v>98</v>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>OLED97G42LW</t>
-        </is>
-      </c>
-      <c r="F131" t="n">
-        <v>4499000</v>
-      </c>
-      <c r="G131" t="n">
-        <v>11304.02</v>
-      </c>
-      <c r="H131" t="n">
-        <v>0</v>
-      </c>
-      <c r="I131" t="n">
-        <v>0</v>
-      </c>
-      <c r="J131" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="K131" t="n">
-        <v>0</v>
-      </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>https://www.mediamarkt.hu/hu/product/_lg-oled97g42lw-oled-evo-smart-tv-4k-tv-ultra-hd-tv-uhd-tv-hdr-webos-thinq-ai-okos-tv-246-cm-1459143.html</t>
-        </is>
-      </c>
-      <c r="M131" t="inlineStr">
-        <is>
-          <t>LG OLED97G42LW OLED evo smart tv,4K TV, Ultra HD TV,uhd TV, HDR,webOS ThinQ AI okos tv, 246 cm</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>Lg</t>
-        </is>
-      </c>
-      <c r="B132" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>OLED M4</t>
-        </is>
-      </c>
-      <c r="D132" t="n">
-        <v>97</v>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>OLED97M49LA</t>
-        </is>
-      </c>
-      <c r="F132" t="n">
-        <v>4999000</v>
-      </c>
-      <c r="G132" t="n">
-        <v>12560.3</v>
-      </c>
-      <c r="H132" t="n">
-        <v>0</v>
-      </c>
-      <c r="I132" t="n">
-        <v>0</v>
-      </c>
-      <c r="J132" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="K132" t="n">
-        <v>0</v>
-      </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t>https://www.mediamarkt.hu/hu/product/_lg-oled97m49la-oled-evo-vezeték-nélküli-smart-tv-4k-tv-ultra-hd-tv-uhd-tv-hdr-webos-thinq-ai-okos-tv-245-cm-1453465.html</t>
-        </is>
-      </c>
-      <c r="M132" t="inlineStr">
-        <is>
-          <t>LG OLED97M49LA OLED evo vezeték nélküli smart tv,4K TV, Ultra HD TV,uhd TV, HDR,webOS ThinQ AI okos tv, 245 cm</t>
         </is>
       </c>
     </row>

</xml_diff>